<commit_message>
3D di dettaglio, visite guidate e istruzioni di montaggio
- Modello 3D rifatto con parti fini: carrelli X, moduli Z (SK16, SC16UU, TR16, BK/BF12),
  motori NEMA23 con giunti, motore R su slitta, catena portacavi, quadro inox con interno
- Viewer: schede Esplora / Come funziona (motori, closed-loop, assi X-Z-R, quadro con
  sportello) / Montaggio (15 fasi animate con frecce)
- ManipMasta_montaggio.pdf con fasi, viteria, coppie e controlli
- Tavole aggiornate: carrello 290x220, slitta 300x250x16 con cuscinetto 6204, coperchio COP-01
- Schemi E01/E02/E03/E05: KM1+KM2 in serie, pull-up ENA 680 ohm, quadro 500x400x250

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9adJsqzSggaSJo74G6Rtt
</commit_message>
<xml_diff>
--- a/bom/ManipMasta_distinta.xlsx
+++ b/bom/ManipMasta_distinta.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>9</v>
@@ -685,7 +685,11 @@
           <t>idem</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2 per albero</t>
+        </is>
+      </c>
       <c r="H6" s="3">
         <f>D6*E6</f>
         <v/>
@@ -847,19 +851,19 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Supporto flangiato inox SUCF204</t>
+          <t>Cuscinetto inox S6204-2RS + seeger DIN 471 Ø20</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>SUCF204 inox foro 20, flangia quadra 4 fori interasse 64</t>
+          <t>S6204-2RS Ø20×47×14 acciaio inox, schermato</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -868,7 +872,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Supporti rullo</t>
+          <t>Nelle sedi delle slitte Z, chiusi da COP-01</t>
         </is>
       </c>
       <c r="H11" s="3">
@@ -2349,7 +2353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2633,7 +2637,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 sp. 12</t>
+          <t>AISI 304 sp. 16</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -2651,11 +2655,11 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>laser, maschiatura, asole motore</t>
+          <t>laser, alesatura sede Ø47 H7, maschiatura, asole motore, bandierina saldata</t>
         </is>
       </c>
       <c r="H7" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="I7" s="3">
         <f>D7*H7</f>
@@ -2675,7 +2679,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 sp. 12</t>
+          <t>AISI 304 sp. 16</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -2693,11 +2697,11 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>laser, maschiatura</t>
+          <t>laser, alesatura sede Ø47 H7, maschiatura, bandierina saldata</t>
         </is>
       </c>
       <c r="H8" s="3" t="n">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="I8" s="3">
         <f>D8*H8</f>
@@ -2707,25 +2711,25 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PIE-01</t>
+          <t>COP-01</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Piastra piede montante</t>
+          <t>Coperchio cuscinetto Ø72</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 sp. 10</t>
+          <t>AISI 304 sp. 5</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Taglio laser + officina</t>
+          <t>Taglio laser + tornitore</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2735,11 +2739,11 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>laser, alesatura Ø20 H7, filetto M12×1 su 2 pezzi</t>
+          <t>laser, tornitura contorno e spallamento Ø47</t>
         </is>
       </c>
       <c r="H9" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I9" s="3">
         <f>D9*H9</f>
@@ -2749,12 +2753,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>STM-01</t>
+          <t>PIE-01</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Flangia motore NEMA23</t>
+          <t>Piastra piede montante</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2777,11 +2781,11 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>laser, foratura</t>
+          <t>laser, alesatura Ø20 H7, filetto M12×1 su 2 pezzi</t>
         </is>
       </c>
       <c r="H10" s="3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I10" s="3">
         <f>D10*H10</f>
@@ -2791,17 +2795,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CTP-01</t>
+          <t>STM-01</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Contropiastra sotto piano</t>
+          <t>Flangia motore NEMA23</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 sp. 5</t>
+          <t>AISI 304 sp. 10</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
@@ -2809,21 +2813,21 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Taglio laser</t>
+          <t>Taglio laser + officina</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Tav. 12</t>
+          <t>Tav. 12 · DXF</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>laser</t>
+          <t>laser, foratura</t>
         </is>
       </c>
       <c r="H11" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I11" s="3">
         <f>D11*H11</f>
@@ -2833,39 +2837,39 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ANC-01</t>
+          <t>CTP-01</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Ancoraggio A1 riferimento</t>
+          <t>Contropiastra sotto piano</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 barra quadra 100</t>
+          <t>AISI 304 sp. 5</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tornitore / fresatore</t>
+          <t>Taglio laser</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Tav. 03</t>
+          <t>Tav. 13</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>fresatura, alesatura Ø20 H7, foro Ø8 H8 trasversale, 4×M8</t>
+          <t>laser</t>
         </is>
       </c>
       <c r="H12" s="3" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="I12" s="3">
         <f>D12*H12</f>
@@ -2875,12 +2879,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ANC-02</t>
+          <t>ANC-01</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ancoraggio A2 asola</t>
+          <t>Ancoraggio A1 riferimento</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2903,11 +2907,11 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>fresatura asola 20 H7×26, foro Ø8 H8, 4×M8</t>
+          <t>fresatura, alesatura Ø20 H7, foro Ø8 H8 trasversale, 4×M8</t>
         </is>
       </c>
       <c r="H13" s="3" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="I13" s="3">
         <f>D13*H13</f>
@@ -2917,12 +2921,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ANC-03</t>
+          <t>ANC-02</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ancoraggio A3/A4 appoggio</t>
+          <t>Ancoraggio A2 asola</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2931,7 +2935,7 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -2945,11 +2949,11 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>fresatura, foro Ø26, 4×M8</t>
+          <t>fresatura asola 20 H7×26, foro Ø8 H8, 4×M8</t>
         </is>
       </c>
       <c r="H14" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="I14" s="3">
         <f>D14*H14</f>
@@ -2959,39 +2963,39 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>PER-01</t>
+          <t>ANC-03</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Perno di centraggio</t>
+          <t>Ancoraggio A3/A4 appoggio</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>AISI 420 temprato (o 304)</t>
+          <t>AISI 304 barra quadra 100</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Tornitore</t>
+          <t>Tornitore / fresatore</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Tav. 04</t>
+          <t>Tav. 03</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>tornitura Ø20 g6, punta conica, foro Ø8 H8 su 2 pezzi</t>
+          <t>fresatura, foro Ø26, 4×M8</t>
         </is>
       </c>
       <c r="H15" s="3" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="I15" s="3">
         <f>D15*H15</f>
@@ -3001,39 +3005,39 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>RUL-01</t>
+          <t>PER-01</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Rullo di laminazione Ø100</t>
+          <t>Perno di centraggio</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 tubo Ø100×3 + testate + perni</t>
+          <t>AISI 420 temprato (o 304)</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Tornitore (rettifica)</t>
+          <t>Tornitore</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Tav. 05</t>
+          <t>Tav. 04</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>saldatura testate, tornitura tra le punte, rettifica e lucidatura Ra≤0,8, cava linguetta, equilibratura</t>
+          <t>tornitura Ø20 g6, punta conica, foro Ø8 H8 su 2 pezzi</t>
         </is>
       </c>
       <c r="H16" s="3" t="n">
-        <v>380</v>
+        <v>35</v>
       </c>
       <c r="I16" s="3">
         <f>D16*H16</f>
@@ -3043,17 +3047,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ASS-X</t>
+          <t>RUL-01</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Albero di sincronismo</t>
+          <t>Rullo di laminazione Ø100</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 Ø16</t>
+          <t>AISI 304 tubo Ø100×3 + testate + perni</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
@@ -3061,21 +3065,21 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Tornitore</t>
+          <t>Tornitore (rettifica)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Tav. 12</t>
+          <t>Tav. 05</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>tornitura sedi Ø15 k6, 2 cave linguetta, estremità Ø14</t>
+          <t>saldatura testate, tornitura tra le punte, rettifica e lucidatura Ra≤0,8, cava linguetta, equilibratura</t>
         </is>
       </c>
       <c r="H17" s="3" t="n">
-        <v>70</v>
+        <v>380</v>
       </c>
       <c r="I17" s="3">
         <f>D17*H17</f>
@@ -3085,21 +3089,21 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DIS-01</t>
+          <t>ASS-X</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Distanziali motore Z 40 mm</t>
+          <t>Albero di sincronismo</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>AISI 304 Ø12 forato</t>
+          <t>AISI 304 Ø16</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -3108,16 +3112,16 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Tav. 12</t>
+          <t>Tav. 13</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>tornitura</t>
+          <t>tornitura sedi Ø15 k6, 2 cave linguetta, estremità Ø14</t>
         </is>
       </c>
       <c r="H18" s="3" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="I18" s="3">
         <f>D18*H18</f>
@@ -3127,39 +3131,39 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>RAS-01</t>
+          <t>DIS-01</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Raschietto rullo</t>
+          <t>Distanziali motore Z 40 mm</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>POM-C alimentare sp. 10</t>
+          <t>AISI 304 Ø12 forato</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Fresatura materie plastiche</t>
+          <t>Tornitore</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Tav. 12</t>
+          <t>Tav. 13</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>fresatura lama 20°, asole</t>
+          <t>tornitura</t>
         </is>
       </c>
       <c r="H19" s="3" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I19" s="3">
         <f>D19*H19</f>
@@ -3169,39 +3173,39 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>QE-01</t>
+          <t>RAS-01</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Cablaggio quadro elettrico + collaudo</t>
+          <t>Raschietto rullo</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>secondo wiring/schemi_elettrici.pdf</t>
+          <t>POM-C alimentare sp. 10</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Quadrista / elettricista</t>
+          <t>Fresatura materie plastiche</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>E01–E05</t>
+          <t>Tav. 13</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>montaggio, cablaggio, prove CEI EN 60204-1, dichiarazione</t>
+          <t>fresatura lama 20°, asole</t>
         </is>
       </c>
       <c r="H20" s="3" t="n">
-        <v>600</v>
+        <v>30</v>
       </c>
       <c r="I20" s="3">
         <f>D20*H20</f>
@@ -3209,17 +3213,59 @@
       </c>
     </row>
     <row r="21">
-      <c r="H21" s="4" t="n"/>
-      <c r="I21" s="4" t="n"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>QE-01</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Cablaggio quadro elettrico + collaudo</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>secondo wiring/schemi_elettrici.pdf</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Quadrista / elettricista</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>E01–E05</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>montaggio, cablaggio, prove CEI EN 60204-1, dichiarazione</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="I21" s="3">
+        <f>D21*H21</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Totale stimato</t>
         </is>
       </c>
-      <c r="I22" s="6">
-        <f>SUM(I2:I20)</f>
+      <c r="I23" s="6">
+        <f>SUM(I2:I21)</f>
         <v/>
       </c>
     </row>
@@ -3266,7 +3312,7 @@
         </is>
       </c>
       <c r="B4" s="8">
-        <f>Artigiani!I22</f>
+        <f>Artigiani!I23</f>
         <v/>
       </c>
     </row>

</xml_diff>